<commit_message>
feat: expand QoR corpus and workbook controls
</commit_message>
<xml_diff>
--- a/artifacts/ENG001-redwood-draft.xlsx
+++ b/artifacts/ENG001-redwood-draft.xlsx
@@ -5,17 +5,25 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Executive Summary" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Reconciliation" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Assumptions" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Findings" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Source Trace" state="visible" r:id="rId8"/>
+    <sheet sheetId="2" name="QoR Waterfall" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Cash Collections" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="AR Aging" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Payer Analysis" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Location Analysis" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="Provider Analysis" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="Service Line" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Collection Curves" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="Assumptions" state="visible" r:id="rId13"/>
+    <sheet sheetId="11" name="Reconciliation" state="visible" r:id="rId14"/>
+    <sheet sheetId="12" name="Findings" state="visible" r:id="rId15"/>
+    <sheet sheetId="13" name="Source Trace" state="visible" r:id="rId16"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="122">
   <si>
     <t>Redwood Quality of Revenue Databook</t>
   </si>
@@ -56,6 +64,183 @@
     <t>Realizable revenue</t>
   </si>
   <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Cash event ID</t>
+  </si>
+  <si>
+    <t>Claim ID</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Payment date</t>
+  </si>
+  <si>
+    <t>Payer</t>
+  </si>
+  <si>
+    <t>ENG001-P001</t>
+  </si>
+  <si>
+    <t>ENG001-C001</t>
+  </si>
+  <si>
+    <t>payer_payment</t>
+  </si>
+  <si>
+    <t>2026-06-10</t>
+  </si>
+  <si>
+    <t>Medicare</t>
+  </si>
+  <si>
+    <t>ENG001-P002</t>
+  </si>
+  <si>
+    <t>ENG001-C002</t>
+  </si>
+  <si>
+    <t>2026-06-29</t>
+  </si>
+  <si>
+    <t>BCBS Texas</t>
+  </si>
+  <si>
+    <t>ENG001-P003</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>unapplied_cash</t>
+  </si>
+  <si>
+    <t>2026-06-30</t>
+  </si>
+  <si>
+    <t>Unapplied</t>
+  </si>
+  <si>
+    <t>Receivable ID</t>
+  </si>
+  <si>
+    <t>Snapshot</t>
+  </si>
+  <si>
+    <t>Age basis</t>
+  </si>
+  <si>
+    <t>Age bucket</t>
+  </si>
+  <si>
+    <t>Balance</t>
+  </si>
+  <si>
+    <t>Valuation snapshot</t>
+  </si>
+  <si>
+    <t>ENG001-AR001:2026-06-30</t>
+  </si>
+  <si>
+    <t>service_date</t>
+  </si>
+  <si>
+    <t>0-30</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>ENG001-AR002:2026-06-30</t>
+  </si>
+  <si>
+    <t>121+</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>LOC-01</t>
+  </si>
+  <si>
+    <t>LOC-02</t>
+  </si>
+  <si>
+    <t>Provider</t>
+  </si>
+  <si>
+    <t>PRV-001</t>
+  </si>
+  <si>
+    <t>PRV-002</t>
+  </si>
+  <si>
+    <t>Service line</t>
+  </si>
+  <si>
+    <t>Cardiology</t>
+  </si>
+  <si>
+    <t>Orthopedics</t>
+  </si>
+  <si>
+    <t>Configured recovery rate</t>
+  </si>
+  <si>
+    <t>A/R balance</t>
+  </si>
+  <si>
+    <t>Expected recovery</t>
+  </si>
+  <si>
+    <t>31-60</t>
+  </si>
+  <si>
+    <t>61-90</t>
+  </si>
+  <si>
+    <t>91-120</t>
+  </si>
+  <si>
+    <t>Method profile</t>
+  </si>
+  <si>
+    <t>redwood-physician-group-qor-draft-v0.1</t>
+  </si>
+  <si>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>0.1.0</t>
+  </si>
+  <si>
+    <t>Professional materiality</t>
+  </si>
+  <si>
+    <t>Unset until approved</t>
+  </si>
+  <si>
+    <t>Recovery methodology</t>
+  </si>
+  <si>
+    <t>Method-profile configured; approval-bound</t>
+  </si>
+  <si>
+    <t>Authoritative editable recovery rates</t>
+  </si>
+  <si>
+    <t>Collection Curves!B2:B6</t>
+  </si>
+  <si>
+    <t>Important</t>
+  </si>
+  <si>
+    <t>Changing the workbook assumptions does not approve a platform Method Profile or release a client work product.</t>
+  </si>
+  <si>
     <t>Control</t>
   </si>
   <si>
@@ -101,30 +286,6 @@
     <t>bf94986286656f63b92f66fc57c5412a219ec14a7e0fc6604d7aba34d9fd5fe2:2; bf94986286656f63b92f66fc57c5412a219ec14a7e0fc6604d7aba34d9fd5fe2:3; 45aed22e980cb357ba709f0da96d3a033b7669da1e9ce3bff1fa9ef88da1044e:2</t>
   </si>
   <si>
-    <t>Method profile</t>
-  </si>
-  <si>
-    <t>redwood-physician-group-qor-draft-v0.1</t>
-  </si>
-  <si>
-    <t>Version</t>
-  </si>
-  <si>
-    <t>0.1.0</t>
-  </si>
-  <si>
-    <t>Professional materiality</t>
-  </si>
-  <si>
-    <t>Unset until approved</t>
-  </si>
-  <si>
-    <t>Recovery methodology</t>
-  </si>
-  <si>
-    <t>Method-profile configured; approval-bound</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
@@ -191,13 +352,13 @@
     <t>Claim</t>
   </si>
   <si>
-    <t>ENG001-C001</t>
+    <t>ENG001-C001:v1</t>
   </si>
   <si>
     <t>8915d58574a70bb9a9058707176d3e3e8061f7e5749f1e7b5e33d31c98ca84ca:3</t>
   </si>
   <si>
-    <t>ENG001-C002</t>
+    <t>ENG001-C002:v1</t>
   </si>
   <si>
     <t>payments.csv</t>
@@ -212,18 +373,9 @@
     <t>CashEvent</t>
   </si>
   <si>
-    <t>ENG001-P001</t>
-  </si>
-  <si>
     <t>cfc655633d1d8c9f558ad2f75e1f329597e57be42c3ec10add578f66065ee9ea:3</t>
   </si>
   <si>
-    <t>ENG001-P002</t>
-  </si>
-  <si>
-    <t>ENG001-P003</t>
-  </si>
-  <si>
     <t>ar_snapshot.csv</t>
   </si>
   <si>
@@ -236,21 +388,16 @@
     <t>Receivable</t>
   </si>
   <si>
-    <t>ENG001-AR001:2026-06-30</t>
-  </si>
-  <si>
     <t>bf94986286656f63b92f66fc57c5412a219ec14a7e0fc6604d7aba34d9fd5fe2:3</t>
-  </si>
-  <si>
-    <t>ENG001-AR002:2026-06-30</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="$#,##0.00;[Red]-$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -285,11 +432,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -633,19 +782,20 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="2" max="2" width="24" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="3"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -653,7 +803,7 @@
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
     </row>
@@ -661,7 +811,7 @@
       <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
     </row>
@@ -669,7 +819,7 @@
       <c r="A6" t="s">
         <v>7</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="1">
         <v>109646.56</v>
       </c>
     </row>
@@ -677,7 +827,7 @@
       <c r="A7" t="s">
         <v>8</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="1">
         <v>69116.88</v>
       </c>
     </row>
@@ -685,7 +835,7 @@
       <c r="A8" t="s">
         <v>9</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="1">
         <v>53527.04</v>
       </c>
     </row>
@@ -693,7 +843,7 @@
       <c r="A9" t="s">
         <v>10</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="1">
         <v>15911.29</v>
       </c>
     </row>
@@ -701,16 +851,420 @@
       <c r="A10" t="s">
         <v>11</v>
       </c>
-      <c r="B10">
-        <v>7102.94</v>
+      <c r="B10" s="1">
+        <f>SUM('Collection Curves'!D2:D6)</f>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="1">
         <f>B8+B10</f>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="2" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="4" width="18" style="1" customWidth="1"/>
+    <col min="5" max="7" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" s="1">
+        <v>53527.04</v>
+      </c>
+      <c r="C2" s="1">
+        <v>52777.04</v>
+      </c>
+      <c r="D2" s="1">
+        <f>B2-C2</f>
+      </c>
+      <c r="E2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F2" t="s">
+        <v>81</v>
+      </c>
+      <c r="G2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" s="1">
+        <v>53205.59</v>
+      </c>
+      <c r="C3" s="1">
+        <v>52134.14</v>
+      </c>
+      <c r="D3" s="1">
+        <f>B3-C3</f>
+      </c>
+      <c r="E3" t="s">
+        <v>80</v>
+      </c>
+      <c r="F3" t="s">
+        <v>81</v>
+      </c>
+      <c r="G3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="1">
+        <v>15911.29</v>
+      </c>
+      <c r="C4" s="1">
+        <v>14506.28</v>
+      </c>
+      <c r="D4" s="1">
+        <f>B4-C4</f>
+      </c>
+      <c r="E4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="4" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="5" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D3" t="s">
+        <v>108</v>
+      </c>
+      <c r="E3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D4" t="s">
+        <v>115</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C5" t="s">
+        <v>116</v>
+      </c>
+      <c r="D5" t="s">
+        <v>115</v>
+      </c>
+      <c r="E5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C6" t="s">
+        <v>99</v>
+      </c>
+      <c r="D6" t="s">
+        <v>115</v>
+      </c>
+      <c r="E6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>117</v>
+      </c>
+      <c r="B7" t="s">
+        <v>118</v>
+      </c>
+      <c r="C7" t="s">
+        <v>119</v>
+      </c>
+      <c r="D7" t="s">
+        <v>120</v>
+      </c>
+      <c r="E7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C8" t="s">
+        <v>121</v>
+      </c>
+      <c r="D8" t="s">
+        <v>120</v>
+      </c>
+      <c r="E8" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -721,104 +1275,59 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="4" width="18" style="2" customWidth="1"/>
-    <col min="5" max="7" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" s="2">
-        <v>53527.04</v>
-      </c>
-      <c r="C2" s="2">
-        <v>52777.04</v>
-      </c>
-      <c r="D2" s="2">
-        <f>B2-C2</f>
-      </c>
-      <c r="E2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1">
+        <f>'Executive Summary'!B6</f>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="2">
-        <v>53205.59</v>
-      </c>
-      <c r="C3" s="2">
-        <v>52134.14</v>
-      </c>
-      <c r="D3" s="2">
-        <f>B3-C3</f>
-      </c>
-      <c r="E3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" t="s">
-        <v>22</v>
-      </c>
-      <c r="G3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="B3" s="1">
+        <f>'Executive Summary'!B7</f>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="2">
-        <v>15911.29</v>
-      </c>
-      <c r="C4" s="2">
-        <v>14506.28</v>
-      </c>
-      <c r="D4" s="2">
-        <f>B4-C4</f>
-      </c>
-      <c r="E4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" t="s">
-        <v>27</v>
+        <v>9</v>
+      </c>
+      <c r="B4" s="1">
+        <f>'Executive Summary'!B8</f>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="1">
+        <f>'Executive Summary'!B10</f>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="1">
+        <f>B4+B5</f>
       </c>
     </row>
   </sheetData>
@@ -829,42 +1338,91 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="18" customWidth="1"/>
+    <col min="1" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="18" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="1">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="1">
+        <v>3205.59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B4" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C4" t="s">
         <v>30</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D4" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="E4" t="s">
         <v>32</v>
       </c>
-      <c r="B3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" t="s">
-        <v>35</v>
+      <c r="F4" s="1">
+        <v>321.45</v>
       </c>
     </row>
   </sheetData>
@@ -875,80 +1433,81 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="4" width="18" customWidth="1"/>
+    <col min="1" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="18" style="1" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>39</v>
       </c>
       <c r="B2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
         <v>40</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>41</v>
       </c>
-      <c r="D2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F2" s="1">
+        <v>6889.77</v>
+      </c>
+      <c r="G2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="1">
+        <v>9021.52</v>
+      </c>
+      <c r="G3" t="s">
         <v>42</v>
-      </c>
-      <c r="C3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5" t="s">
-        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -959,146 +1518,260 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="5" width="18" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="1">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="1">
+        <v>3205.59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="1">
+        <v>321.45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="1">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="1">
+        <v>49646.56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" s="1">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>50</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B3" s="1">
+        <v>49646.56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="B2" s="1">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3" s="1">
+        <v>49646.56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" style="4" customWidth="1"/>
+    <col min="3" max="4" width="18" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="4">
+        <v>0.9</v>
+      </c>
+      <c r="C2" s="1">
+        <f>SUMIFS('AR Aging'!F:F,'AR Aging'!E:E,A2,'AR Aging'!G:G,"Active")</f>
+      </c>
+      <c r="D2" s="1">
+        <f>B2*C2</f>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>57</v>
       </c>
-      <c r="E2" t="s">
+      <c r="B3" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="C3" s="1">
+        <f>SUMIFS('AR Aging'!F:F,'AR Aging'!E:E,A3,'AR Aging'!G:G,"Active")</f>
+      </c>
+      <c r="D3" s="1">
+        <f>B3*C3</f>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B4" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="C4" s="1">
+        <f>SUMIFS('AR Aging'!F:F,'AR Aging'!E:E,A4,'AR Aging'!G:G,"Active")</f>
+      </c>
+      <c r="D4" s="1">
+        <f>B4*C4</f>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>59</v>
       </c>
-      <c r="D3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B4" t="s">
-        <v>62</v>
-      </c>
-      <c r="C4" t="s">
-        <v>63</v>
-      </c>
-      <c r="D4" t="s">
-        <v>64</v>
-      </c>
-      <c r="E4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D5" t="s">
-        <v>64</v>
-      </c>
-      <c r="E5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B5" s="4">
+        <v>0.3</v>
+      </c>
+      <c r="C5" s="1">
+        <f>SUMIFS('AR Aging'!F:F,'AR Aging'!E:E,A5,'AR Aging'!G:G,"Active")</f>
+      </c>
+      <c r="D5" s="1">
+        <f>B5*C5</f>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>61</v>
-      </c>
-      <c r="B6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C6" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E6" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>69</v>
-      </c>
-      <c r="B7" t="s">
-        <v>70</v>
-      </c>
-      <c r="C7" t="s">
-        <v>71</v>
-      </c>
-      <c r="D7" t="s">
-        <v>72</v>
-      </c>
-      <c r="E7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>69</v>
-      </c>
-      <c r="B8" t="s">
-        <v>70</v>
-      </c>
-      <c r="C8" t="s">
-        <v>74</v>
-      </c>
-      <c r="D8" t="s">
-        <v>72</v>
-      </c>
-      <c r="E8" t="s">
-        <v>75</v>
+        <v>44</v>
+      </c>
+      <c r="B6" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="C6" s="1">
+        <f>SUMIFS('AR Aging'!F:F,'AR Aging'!E:E,A6,'AR Aging'!G:G,"Active")</f>
+      </c>
+      <c r="D6" s="1">
+        <f>B6*C6</f>
       </c>
     </row>
   </sheetData>

</xml_diff>